<commit_message>
Added ACCA AFM file
</commit_message>
<xml_diff>
--- a/myprojects/ExelProj/RestoreX_EFP.xlsx
+++ b/myprojects/ExelProj/RestoreX_EFP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\inanj\Documents\GitHub\inakm.github.io\myprojects\ExelProj\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D85DFF-D208-46A3-8CD8-DA710FDE2DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{464AF83F-C59F-4A6C-9A7C-A1F82DB17E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{7C2FD2EF-2EBC-42C0-8B2D-B63F3F4A082A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="2" xr2:uid="{7C2FD2EF-2EBC-42C0-8B2D-B63F3F4A082A}"/>
   </bookViews>
   <sheets>
     <sheet name="HOME" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="164">
   <si>
     <t>🔒 RestoreX</t>
   </si>
@@ -156,9 +156,6 @@
     <t>Total Estimated One-Time Cost</t>
   </si>
   <si>
-    <t>MONTHLY OPERATING COSTS (Recurring )</t>
-  </si>
-  <si>
     <t xml:space="preserve">Monthly Cost </t>
   </si>
   <si>
@@ -172,9 +169,6 @@
   </si>
   <si>
     <t>Database</t>
-  </si>
-  <si>
-    <t>Redis Cache</t>
   </si>
   <si>
     <t>CDN / Static Assets</t>
@@ -647,6 +641,75 @@
   <si>
     <t>5-15</t>
   </si>
+  <si>
+    <t>DigitalOcean</t>
+  </si>
+  <si>
+    <t>Automated Backups</t>
+  </si>
+  <si>
+    <t>Discord</t>
+  </si>
+  <si>
+    <t>Gitbook, Notion</t>
+  </si>
+  <si>
+    <t>Cloudflare</t>
+  </si>
+  <si>
+    <t>Bigrock</t>
+  </si>
+  <si>
+    <t>UptimeRobot</t>
+  </si>
+  <si>
+    <t>MONTHLY OPERATING COSTS - Growth Phase</t>
+  </si>
+  <si>
+    <t>$22 - $43/m</t>
+  </si>
+  <si>
+    <t>MONTHLY OPERATING COSTS - Lean Phase</t>
+  </si>
+  <si>
+    <t>Resend</t>
+  </si>
+  <si>
+    <t>$72 - $150/m</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Monthly Costs</t>
+  </si>
+  <si>
+    <t>Avg. Revenue/Subscriber</t>
+  </si>
+  <si>
+    <t>Break-Even Subscribers</t>
+  </si>
+  <si>
+    <t>Lean Phase</t>
+  </si>
+  <si>
+    <t>Growth Phase</t>
+  </si>
+  <si>
+    <t>Full Scale</t>
+  </si>
+  <si>
+    <t>Blended Average</t>
+  </si>
+  <si>
+    <t>Mix</t>
+  </si>
+  <si>
+    <t>Contribution</t>
+  </si>
+  <si>
+    <t>SUM</t>
+  </si>
 </sst>
 </file>
 
@@ -752,7 +815,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -896,12 +959,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -947,161 +1021,167 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1109,11 +1189,32 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1140,33 +1241,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1886,91 +1990,91 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="32"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="36"/>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B3" s="33"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="35"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="39"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B4" s="33"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="35"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="39"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B5" s="33"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="35"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="39"/>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="38"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="42"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="41"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="44"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="44"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="47"/>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="48"/>
       <c r="C9" s="48"/>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="I10" s="40" t="s">
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="I10" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="J10" s="40"/>
-      <c r="K10" s="40"/>
-      <c r="L10" s="40"/>
-      <c r="M10" s="40"/>
-      <c r="N10" s="40"/>
-      <c r="O10" s="40"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="30"/>
     </row>
     <row r="11" spans="2:15" ht="7.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="48"/>
@@ -1981,25 +2085,25 @@
       <c r="G11" s="48"/>
     </row>
     <row r="12" spans="2:15" ht="87" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="45" t="s">
-        <v>141</v>
-      </c>
-      <c r="C12" s="45"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
+      <c r="B12" s="31" t="s">
+        <v>139</v>
+      </c>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
     </row>
     <row r="13" spans="2:15" ht="6.6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="2:15" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="45" t="s">
+      <c r="B14" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B16" s="55" t="s">
@@ -2020,52 +2124,52 @@
       <c r="G17" s="24"/>
     </row>
     <row r="18" spans="2:16" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="59"/>
-      <c r="D18" s="59"/>
-      <c r="E18" s="59"/>
-      <c r="F18" s="59"/>
-      <c r="G18" s="60"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="29"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B20" s="40" t="s">
+      <c r="B20" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="40"/>
-      <c r="D20" s="40"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="I20" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="J20" s="40"/>
-      <c r="K20" s="40"/>
-      <c r="L20" s="40"/>
-      <c r="M20" s="40"/>
-      <c r="N20" s="40"/>
-      <c r="O20" s="40"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="I20" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
+      <c r="M20" s="30"/>
+      <c r="N20" s="30"/>
+      <c r="O20" s="30"/>
     </row>
     <row r="22" spans="2:16" ht="218.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="45" t="s">
+      <c r="B22" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="I22" s="45" t="s">
-        <v>72</v>
-      </c>
-      <c r="J22" s="46"/>
-      <c r="K22" s="46"/>
-      <c r="L22" s="46"/>
-      <c r="M22" s="46"/>
-      <c r="N22" s="46"/>
-      <c r="O22" s="46"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="31"/>
+      <c r="I22" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+      <c r="L22" s="32"/>
+      <c r="M22" s="32"/>
+      <c r="N22" s="32"/>
+      <c r="O22" s="32"/>
     </row>
     <row r="23" spans="2:16" ht="7.8" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="24" spans="2:16" x14ac:dyDescent="0.3">
@@ -2097,36 +2201,36 @@
       <c r="G26" s="54"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B30" s="47" t="s">
-        <v>73</v>
-      </c>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="47"/>
-      <c r="G30" s="47"/>
-      <c r="H30" s="47"/>
-      <c r="I30" s="47"/>
-      <c r="J30" s="47"/>
-      <c r="K30" s="47"/>
-      <c r="L30" s="47"/>
-      <c r="M30" s="47"/>
-      <c r="N30" s="47"/>
-      <c r="O30" s="47"/>
-      <c r="P30" s="47"/>
+      <c r="B30" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
+      <c r="K30" s="33"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="33"/>
+      <c r="N30" s="33"/>
+      <c r="O30" s="33"/>
+      <c r="P30" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="B2:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B9:C9"/>
     <mergeCell ref="B18:G18"/>
     <mergeCell ref="I10:O10"/>
     <mergeCell ref="I20:O20"/>
     <mergeCell ref="I22:O22"/>
     <mergeCell ref="B30:P30"/>
-    <mergeCell ref="B2:G5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B9:C9"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B22:G22"/>
     <mergeCell ref="B24:G24"/>
@@ -2145,7 +2249,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DEFCF0A-B28A-4F57-8452-DFE5A338C55E}">
-  <dimension ref="B2:P33"/>
+  <dimension ref="B2:P49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.6640625" customWidth="1"/>
@@ -2153,551 +2257,747 @@
     <col min="9" max="9" width="9.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="32"/>
-    </row>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B3" s="33"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="35"/>
-    </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B4" s="33"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="35"/>
-    </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B5" s="33"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="35"/>
-    </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B6" s="36" t="s">
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="36"/>
+    </row>
+    <row r="3" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B3" s="37"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="39"/>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="39"/>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B5" s="37"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="39"/>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B6" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="38"/>
-    </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B7" s="39" t="s">
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="42"/>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B7" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="41"/>
-    </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B8" s="42" t="s">
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="44"/>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B8" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="44"/>
-    </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B10" s="69" t="s">
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="47"/>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B10" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="69"/>
-      <c r="D10" s="69"/>
-      <c r="E10" s="69"/>
-      <c r="F10" s="69"/>
-      <c r="G10" s="69"/>
-      <c r="I10" s="73" t="s">
+      <c r="C10" s="68"/>
+      <c r="D10" s="68"/>
+      <c r="E10" s="68"/>
+      <c r="F10" s="68"/>
+      <c r="G10" s="68"/>
+      <c r="I10" s="63" t="s">
+        <v>42</v>
+      </c>
+      <c r="J10" s="63"/>
+      <c r="K10" s="63"/>
+      <c r="L10" s="63"/>
+      <c r="M10" s="63"/>
+      <c r="N10" s="63"/>
+      <c r="O10" s="63"/>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B11" s="69" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="69"/>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B12" s="65" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="65"/>
+      <c r="D12" s="71" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="71"/>
+      <c r="F12" s="70">
+        <v>15</v>
+      </c>
+      <c r="G12" s="70"/>
+      <c r="I12" s="64" t="s">
+        <v>43</v>
+      </c>
+      <c r="J12" s="64"/>
+      <c r="K12" s="64"/>
+      <c r="L12" s="64"/>
+      <c r="M12" s="64"/>
+      <c r="N12" s="64"/>
+      <c r="O12" s="64"/>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B13" s="65" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="65"/>
+      <c r="D13" s="71" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="71"/>
+      <c r="F13" s="70">
+        <v>10</v>
+      </c>
+      <c r="G13" s="70"/>
+      <c r="I13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="73"/>
-      <c r="K10" s="73"/>
-      <c r="L10" s="73"/>
-      <c r="M10" s="73"/>
-      <c r="N10" s="73"/>
-      <c r="O10" s="73"/>
-    </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B11" s="29" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="G11" s="29"/>
-      <c r="I11" s="74" t="s">
+      <c r="J13" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J11" s="74"/>
-      <c r="K11" s="74"/>
-      <c r="L11" s="74"/>
-      <c r="M11" s="74"/>
-      <c r="N11" s="74"/>
-      <c r="O11" s="74"/>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B12" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="25"/>
-      <c r="D12" s="67" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="67"/>
-      <c r="F12" s="68">
-        <v>15</v>
-      </c>
-      <c r="G12" s="68"/>
-      <c r="I12" s="4" t="s">
+      <c r="K13" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="L13" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B14" s="65" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="65"/>
+      <c r="D14" s="71" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="71"/>
+      <c r="F14" s="70">
+        <v>0</v>
+      </c>
+      <c r="G14" s="70"/>
+      <c r="I14" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="J14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K14" s="6">
+        <v>0</v>
+      </c>
+      <c r="L14" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="M14" s="25"/>
+      <c r="N14" s="25"/>
+      <c r="O14" s="25"/>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B15" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="65"/>
+      <c r="D15" s="71" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" s="71"/>
+      <c r="F15" s="70">
+        <v>0</v>
+      </c>
+      <c r="G15" s="70"/>
+      <c r="I15" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="L12" s="75" t="s">
-        <v>31</v>
-      </c>
-      <c r="M12" s="75"/>
-      <c r="N12" s="75"/>
-      <c r="O12" s="75"/>
-    </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B13" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="25"/>
-      <c r="D13" s="67" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="67"/>
-      <c r="F13" s="68">
-        <v>10</v>
-      </c>
-      <c r="G13" s="68"/>
-      <c r="I13" s="5" t="s">
+      <c r="J15" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="K15" s="6">
+        <v>3.99</v>
+      </c>
+      <c r="L15" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="M15" s="25"/>
+      <c r="N15" s="25"/>
+      <c r="O15" s="25"/>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B16" s="65" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="65"/>
+      <c r="D16" s="71" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="71"/>
+      <c r="F16" s="70">
+        <v>0</v>
+      </c>
+      <c r="G16" s="70"/>
+      <c r="I16" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J16" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K16" s="6">
+        <v>8.99</v>
+      </c>
+      <c r="L16" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="M16" s="26"/>
+      <c r="N16" s="26"/>
+      <c r="O16" s="26"/>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B17" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="65"/>
+      <c r="D17" s="71" t="s">
+        <v>21</v>
+      </c>
+      <c r="E17" s="71"/>
+      <c r="F17" s="70">
+        <v>50</v>
+      </c>
+      <c r="G17" s="70"/>
+      <c r="I17" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K17" s="6">
+        <v>24.99</v>
+      </c>
+      <c r="L17" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B18" s="65" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="65"/>
+      <c r="D18" s="71" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="71"/>
+      <c r="F18" s="70">
         <v>0</v>
       </c>
-      <c r="L13" s="46" t="s">
-        <v>59</v>
-      </c>
-      <c r="M13" s="46"/>
-      <c r="N13" s="46"/>
-      <c r="O13" s="46"/>
-    </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B14" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="67" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="67"/>
-      <c r="F14" s="68">
-        <v>0</v>
-      </c>
-      <c r="G14" s="68"/>
-      <c r="I14" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="K14" s="6">
-        <v>3.99</v>
-      </c>
-      <c r="L14" s="46" t="s">
-        <v>60</v>
-      </c>
-      <c r="M14" s="46"/>
-      <c r="N14" s="46"/>
-      <c r="O14" s="46"/>
-    </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B15" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="25"/>
-      <c r="D15" s="67" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" s="67"/>
-      <c r="F15" s="68">
-        <v>0</v>
-      </c>
-      <c r="G15" s="68"/>
-      <c r="I15" s="5" t="s">
+      <c r="G18" s="70"/>
+      <c r="I18" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J18" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="K15" s="6">
-        <v>8.99</v>
-      </c>
-      <c r="L15" s="48" t="s">
+      <c r="K18" s="6">
+        <v>4</v>
+      </c>
+      <c r="L18" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="M15" s="48"/>
-      <c r="N15" s="48"/>
-      <c r="O15" s="48"/>
-    </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B16" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="25"/>
-      <c r="D16" s="67" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" s="67"/>
-      <c r="F16" s="68">
-        <v>0</v>
-      </c>
-      <c r="G16" s="68"/>
-      <c r="I16" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="K16" s="6">
-        <v>24.99</v>
-      </c>
-      <c r="L16" s="46" t="s">
-        <v>62</v>
-      </c>
-      <c r="M16" s="46"/>
-      <c r="N16" s="46"/>
-      <c r="O16" s="46"/>
-      <c r="P16" s="46"/>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B17" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="25"/>
-      <c r="D17" s="67" t="s">
-        <v>21</v>
-      </c>
-      <c r="E17" s="67"/>
-      <c r="F17" s="68">
-        <v>50</v>
-      </c>
-      <c r="G17" s="68"/>
-      <c r="I17" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="K17" s="6">
-        <v>89.99</v>
-      </c>
-      <c r="L17" s="46" t="s">
-        <v>63</v>
-      </c>
-      <c r="M17" s="46"/>
-      <c r="N17" s="46"/>
-      <c r="O17" s="46"/>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="67" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="67"/>
-      <c r="F18" s="68">
-        <v>0</v>
-      </c>
-      <c r="G18" s="68"/>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B19" s="71" t="s">
+      <c r="M18" s="25"/>
+      <c r="N18" s="25"/>
+      <c r="O18" s="25"/>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B19" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="71"/>
-      <c r="D19" s="71"/>
-      <c r="E19" s="71"/>
-      <c r="F19" s="70">
+      <c r="C19" s="67"/>
+      <c r="D19" s="67"/>
+      <c r="E19" s="67"/>
+      <c r="F19" s="66">
         <f>SUM(F12:G18)</f>
         <v>75</v>
       </c>
-      <c r="G19" s="70"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B21" s="69" t="s">
+      <c r="G19" s="66"/>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B21" s="68" t="s">
+        <v>150</v>
+      </c>
+      <c r="C21" s="68"/>
+      <c r="D21" s="68"/>
+      <c r="E21" s="68"/>
+      <c r="F21" s="68"/>
+      <c r="G21" s="68"/>
+      <c r="I21" s="68" t="s">
+        <v>148</v>
+      </c>
+      <c r="J21" s="68"/>
+      <c r="K21" s="68"/>
+      <c r="L21" s="68"/>
+      <c r="M21" s="68"/>
+      <c r="N21" s="68"/>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B22" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="69"/>
+      <c r="D22" s="69" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="69"/>
+      <c r="F22" s="69" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="69"/>
-      <c r="D21" s="69"/>
-      <c r="E21" s="69"/>
-      <c r="F21" s="69"/>
-      <c r="G21" s="69"/>
-      <c r="I21" s="73" t="s">
+      <c r="G22" s="69"/>
+      <c r="I22" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="J22" s="69"/>
+      <c r="K22" s="69" t="s">
+        <v>68</v>
+      </c>
+      <c r="L22" s="69"/>
+      <c r="M22" s="69" t="s">
+        <v>29</v>
+      </c>
+      <c r="N22" s="69"/>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B23" s="65" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="65"/>
+      <c r="D23" s="58" t="s">
+        <v>141</v>
+      </c>
+      <c r="E23" s="59"/>
+      <c r="F23" s="99">
+        <v>24</v>
+      </c>
+      <c r="G23" s="100"/>
+      <c r="I23" s="65" t="s">
+        <v>32</v>
+      </c>
+      <c r="J23" s="65"/>
+      <c r="K23" s="58" t="s">
+        <v>141</v>
+      </c>
+      <c r="L23" s="59"/>
+      <c r="M23" s="99">
+        <v>96</v>
+      </c>
+      <c r="N23" s="100"/>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B24" s="65" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="65"/>
+      <c r="D24" s="58" t="s">
+        <v>141</v>
+      </c>
+      <c r="E24" s="59"/>
+      <c r="F24" s="99">
+        <v>0</v>
+      </c>
+      <c r="G24" s="100"/>
+      <c r="I24" s="65" t="s">
+        <v>33</v>
+      </c>
+      <c r="J24" s="65"/>
+      <c r="K24" s="58" t="s">
+        <v>141</v>
+      </c>
+      <c r="L24" s="59"/>
+      <c r="M24" s="99">
+        <v>0</v>
+      </c>
+      <c r="N24" s="100"/>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B25" s="75" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" s="76"/>
+      <c r="D25" s="58" t="s">
+        <v>141</v>
+      </c>
+      <c r="E25" s="59"/>
+      <c r="F25" s="99">
+        <f>F23*20%</f>
+        <v>4.8000000000000007</v>
+      </c>
+      <c r="G25" s="100"/>
+      <c r="I25" s="75" t="s">
+        <v>142</v>
+      </c>
+      <c r="J25" s="76"/>
+      <c r="K25" s="58" t="s">
+        <v>141</v>
+      </c>
+      <c r="L25" s="59"/>
+      <c r="M25" s="99">
+        <f>M23*20%</f>
+        <v>19.200000000000003</v>
+      </c>
+      <c r="N25" s="100"/>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B26" s="65" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="65"/>
+      <c r="D26" s="58" t="s">
+        <v>145</v>
+      </c>
+      <c r="E26" s="59"/>
+      <c r="F26" s="99">
+        <v>0</v>
+      </c>
+      <c r="G26" s="100"/>
+      <c r="I26" s="65" t="s">
+        <v>34</v>
+      </c>
+      <c r="J26" s="65"/>
+      <c r="K26" s="58" t="s">
+        <v>145</v>
+      </c>
+      <c r="L26" s="59"/>
+      <c r="M26" s="99">
+        <v>0</v>
+      </c>
+      <c r="N26" s="100"/>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B27" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="58" t="s">
+        <v>146</v>
+      </c>
+      <c r="E27" s="59"/>
+      <c r="F27" s="99">
+        <v>15</v>
+      </c>
+      <c r="G27" s="100"/>
+      <c r="I27" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J27" s="2"/>
+      <c r="K27" s="58" t="s">
+        <v>146</v>
+      </c>
+      <c r="L27" s="59"/>
+      <c r="M27" s="99">
+        <v>15</v>
+      </c>
+      <c r="N27" s="100"/>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B28" s="65" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="65"/>
+      <c r="D28" s="58" t="s">
+        <v>147</v>
+      </c>
+      <c r="E28" s="59"/>
+      <c r="F28" s="99">
+        <v>0</v>
+      </c>
+      <c r="G28" s="100"/>
+      <c r="I28" s="65" t="s">
+        <v>36</v>
+      </c>
+      <c r="J28" s="65"/>
+      <c r="K28" s="58" t="s">
+        <v>147</v>
+      </c>
+      <c r="L28" s="59"/>
+      <c r="M28" s="99">
+        <v>0</v>
+      </c>
+      <c r="N28" s="100"/>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B29" s="65" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="65"/>
+      <c r="D29" s="58" t="s">
+        <v>151</v>
+      </c>
+      <c r="E29" s="59"/>
+      <c r="F29" s="99">
+        <v>0</v>
+      </c>
+      <c r="G29" s="100"/>
+      <c r="I29" s="65" t="s">
+        <v>37</v>
+      </c>
+      <c r="J29" s="65"/>
+      <c r="K29" s="58" t="s">
+        <v>151</v>
+      </c>
+      <c r="L29" s="59"/>
+      <c r="M29" s="99">
+        <v>20</v>
+      </c>
+      <c r="N29" s="100"/>
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B30" s="65" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="65"/>
+      <c r="D30" s="58" t="s">
+        <v>143</v>
+      </c>
+      <c r="E30" s="59"/>
+      <c r="F30" s="99">
+        <v>0</v>
+      </c>
+      <c r="G30" s="100"/>
+      <c r="I30" s="65" t="s">
+        <v>38</v>
+      </c>
+      <c r="J30" s="65"/>
+      <c r="K30" s="58" t="s">
+        <v>143</v>
+      </c>
+      <c r="L30" s="59"/>
+      <c r="M30" s="99">
+        <v>0</v>
+      </c>
+      <c r="N30" s="100"/>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B31" s="65" t="s">
+        <v>39</v>
+      </c>
+      <c r="C31" s="65"/>
+      <c r="D31" s="58" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" s="59"/>
+      <c r="F31" s="99">
+        <v>0</v>
+      </c>
+      <c r="G31" s="100"/>
+      <c r="I31" s="65" t="s">
+        <v>39</v>
+      </c>
+      <c r="J31" s="65"/>
+      <c r="K31" s="58" t="s">
+        <v>144</v>
+      </c>
+      <c r="L31" s="59"/>
+      <c r="M31" s="99">
+        <v>0</v>
+      </c>
+      <c r="N31" s="100"/>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B32" s="72" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="101"/>
+      <c r="D32" s="101"/>
+      <c r="E32" s="73"/>
+      <c r="F32" s="99">
+        <f>SUM(F23:G31)</f>
+        <v>43.8</v>
+      </c>
+      <c r="G32" s="100"/>
+      <c r="I32" s="72" t="s">
+        <v>40</v>
+      </c>
+      <c r="J32" s="101"/>
+      <c r="K32" s="101"/>
+      <c r="L32" s="73"/>
+      <c r="M32" s="99">
+        <f>SUM(M23:N31)</f>
+        <v>150.19999999999999</v>
+      </c>
+      <c r="N32" s="100"/>
+    </row>
+    <row r="33" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B33" s="62" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="62"/>
+      <c r="D33" s="62"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="99" t="s">
+        <v>149</v>
+      </c>
+      <c r="G33" s="100"/>
+      <c r="I33" s="62" t="s">
+        <v>41</v>
+      </c>
+      <c r="J33" s="62"/>
+      <c r="K33" s="62"/>
+      <c r="L33" s="62"/>
+      <c r="M33" s="99" t="s">
+        <v>152</v>
+      </c>
+      <c r="N33" s="100"/>
+    </row>
+    <row r="35" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B35" s="63" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="63"/>
+      <c r="D35" s="63"/>
+      <c r="E35" s="63"/>
+      <c r="F35" s="63"/>
+      <c r="G35" s="63"/>
+      <c r="H35" s="63"/>
+    </row>
+    <row r="37" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B37" s="60" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37" s="60"/>
+      <c r="D37" s="60"/>
+      <c r="E37" s="60"/>
+      <c r="F37" s="60"/>
+      <c r="G37" s="60"/>
+      <c r="H37" s="60"/>
+    </row>
+    <row r="38" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B38" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="J21" s="73"/>
-      <c r="K21" s="73"/>
-      <c r="L21" s="73"/>
-      <c r="M21" s="73"/>
-      <c r="N21" s="73"/>
-      <c r="O21" s="73"/>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B22" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="G22" s="29"/>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B23" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="C23" s="25"/>
-      <c r="D23" s="63"/>
-      <c r="E23" s="64"/>
-      <c r="F23" s="63"/>
-      <c r="G23" s="64"/>
-      <c r="I23" s="76" t="s">
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+    </row>
+    <row r="40" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B40" s="61" t="s">
         <v>66</v>
       </c>
-      <c r="J23" s="76"/>
-      <c r="K23" s="76"/>
-      <c r="L23" s="76"/>
-      <c r="M23" s="76"/>
-      <c r="N23" s="76"/>
-      <c r="O23" s="76"/>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B24" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="25"/>
-      <c r="D24" s="63"/>
-      <c r="E24" s="64"/>
-      <c r="F24" s="63"/>
-      <c r="G24" s="64"/>
-      <c r="I24" s="46" t="s">
+      <c r="C40" s="61"/>
+      <c r="D40" s="61"/>
+      <c r="E40" s="61"/>
+      <c r="F40" s="61"/>
+      <c r="G40" s="61"/>
+      <c r="H40" s="61"/>
+    </row>
+    <row r="41" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B41" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="J24" s="46"/>
-      <c r="K24" s="46"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="46"/>
-      <c r="N24" s="46"/>
-      <c r="O24" s="46"/>
-    </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B25" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="63"/>
-      <c r="E25" s="64"/>
-      <c r="F25" s="63"/>
-      <c r="G25" s="64"/>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B26" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C26" s="25"/>
-      <c r="D26" s="63"/>
-      <c r="E26" s="64"/>
-      <c r="F26" s="63"/>
-      <c r="G26" s="64"/>
-      <c r="I26" s="75" t="s">
-        <v>68</v>
-      </c>
-      <c r="J26" s="75"/>
-      <c r="K26" s="75"/>
-      <c r="L26" s="75"/>
-      <c r="M26" s="75"/>
-      <c r="N26" s="75"/>
-      <c r="O26" s="75"/>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B27" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="63"/>
-      <c r="E27" s="64"/>
-      <c r="F27" s="63"/>
-      <c r="G27" s="64"/>
-      <c r="I27" s="46" t="s">
-        <v>69</v>
-      </c>
-      <c r="J27" s="46"/>
-      <c r="K27" s="46"/>
-      <c r="L27" s="46"/>
-      <c r="M27" s="46"/>
-      <c r="N27" s="46"/>
-      <c r="O27" s="46"/>
-    </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B28" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="63"/>
-      <c r="E28" s="64"/>
-      <c r="F28" s="63"/>
-      <c r="G28" s="64"/>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B29" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="C29" s="25"/>
-      <c r="D29" s="63"/>
-      <c r="E29" s="64"/>
-      <c r="F29" s="63"/>
-      <c r="G29" s="64"/>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B30" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="C30" s="25"/>
-      <c r="D30" s="63"/>
-      <c r="E30" s="64"/>
-      <c r="F30" s="63"/>
-      <c r="G30" s="64"/>
-    </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B31" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="C31" s="25"/>
-      <c r="D31" s="63"/>
-      <c r="E31" s="64"/>
-      <c r="F31" s="63"/>
-      <c r="G31" s="64"/>
-    </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B32" s="61" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" s="62"/>
-      <c r="D32" s="65"/>
-      <c r="E32" s="66"/>
-      <c r="F32" s="63"/>
-      <c r="G32" s="64"/>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B33" s="72" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" s="72"/>
-      <c r="D33" s="72"/>
-      <c r="E33" s="72"/>
-      <c r="F33" s="63"/>
-      <c r="G33" s="64"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B49" s="93"/>
+      <c r="C49" s="93"/>
+      <c r="D49" s="93"/>
+      <c r="E49" s="93"/>
+      <c r="F49" s="93"/>
+      <c r="G49" s="93"/>
     </row>
   </sheetData>
-  <mergeCells count="78">
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="I27:O27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="I23:O23"/>
-    <mergeCell ref="I26:O26"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="I24:O24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="I10:O10"/>
-    <mergeCell ref="I11:O11"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="L14:O14"/>
-    <mergeCell ref="L15:O15"/>
-    <mergeCell ref="L16:P16"/>
-    <mergeCell ref="L17:O17"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="I21:O21"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B2:G5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B10:G10"/>
+  <mergeCells count="108">
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="I33:L33"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="I32:L32"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="I21:N21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="B31:C31"/>
     <mergeCell ref="F33:G33"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D11:E11"/>
@@ -2714,12 +3014,56 @@
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="F13:G13"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B2:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="I10:O10"/>
+    <mergeCell ref="I12:O12"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B40:H40"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="B38:H38"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="B41:H41"/>
+    <mergeCell ref="D27:E27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2728,7 +3072,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{739042F5-02A3-4835-AF23-494405E7D033}">
-  <dimension ref="B2:N26"/>
+  <dimension ref="B2:P35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.109375" customWidth="1"/>
@@ -2737,117 +3081,118 @@
     <col min="7" max="7" width="19.21875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="2.109375" customWidth="1"/>
     <col min="14" max="14" width="16.5546875" customWidth="1"/>
+    <col min="16" max="16" width="11.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="32"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="36"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B3" s="33"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="35"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="39"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B4" s="33"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="35"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="39"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B5" s="33"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="35"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="39"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="38"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="42"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="41"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="44"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="44"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="47"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B10" s="40" t="s">
-        <v>74</v>
-      </c>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
+      <c r="B10" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="74" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
+      <c r="F12" s="74"/>
+      <c r="G12" s="74"/>
+      <c r="I12" s="74" t="s">
+        <v>77</v>
+      </c>
+      <c r="J12" s="74"/>
+      <c r="K12" s="74"/>
+      <c r="L12" s="74"/>
+      <c r="M12" s="74"/>
+      <c r="N12" s="74"/>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B13" s="103" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="104" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="104"/>
+      <c r="E13" s="104" t="s">
         <v>80</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="I12" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="J12" s="28"/>
-      <c r="K12" s="28"/>
-      <c r="L12" s="28"/>
-      <c r="M12" s="28"/>
-      <c r="N12" s="28"/>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="29" t="s">
+      <c r="F13" s="104"/>
+      <c r="G13" s="103" t="s">
         <v>81</v>
       </c>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29" t="s">
-        <v>82</v>
-      </c>
-      <c r="F13" s="29"/>
-      <c r="G13" s="4" t="s">
-        <v>83</v>
-      </c>
       <c r="I13" s="48" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J13" s="48"/>
       <c r="K13" s="48"/>
@@ -2857,185 +3202,237 @@
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C14" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="F14" s="27"/>
+        <v>83</v>
+      </c>
+      <c r="C14" s="65" t="s">
+        <v>90</v>
+      </c>
+      <c r="D14" s="65"/>
+      <c r="E14" s="75" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" s="76"/>
       <c r="G14" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="I14" s="46" t="s">
-        <v>76</v>
-      </c>
-      <c r="J14" s="46"/>
-      <c r="K14" s="46"/>
-      <c r="L14" s="46"/>
-      <c r="M14" s="46"/>
-      <c r="N14" s="46"/>
+        <v>103</v>
+      </c>
+      <c r="I14" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+      <c r="L14" s="32"/>
+      <c r="M14" s="32"/>
+      <c r="N14" s="32"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" s="65" t="s">
         <v>91</v>
       </c>
-      <c r="C15" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="79" t="s">
-        <v>142</v>
-      </c>
-      <c r="F15" s="80"/>
+      <c r="D15" s="65"/>
+      <c r="E15" s="77" t="s">
+        <v>140</v>
+      </c>
+      <c r="F15" s="78"/>
       <c r="G15" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="I15" s="46" t="s">
-        <v>77</v>
-      </c>
-      <c r="J15" s="46"/>
-      <c r="K15" s="46"/>
-      <c r="L15" s="46"/>
-      <c r="M15" s="46"/>
-      <c r="N15" s="46"/>
+        <v>104</v>
+      </c>
+      <c r="I15" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="J15" s="32"/>
+      <c r="K15" s="32"/>
+      <c r="L15" s="32"/>
+      <c r="M15" s="32"/>
+      <c r="N15" s="32"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B16" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="65" t="s">
+        <v>92</v>
+      </c>
+      <c r="D16" s="65"/>
+      <c r="E16" s="75" t="s">
+        <v>97</v>
+      </c>
+      <c r="F16" s="76"/>
+      <c r="G16" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="I16" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+      <c r="L16" s="32"/>
+      <c r="M16" s="32"/>
+      <c r="N16" s="32"/>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B17" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="65" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" s="65"/>
+      <c r="E17" s="75" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" s="76"/>
+      <c r="G17" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B18" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C18" s="65" t="s">
         <v>94</v>
       </c>
-      <c r="D16" s="25"/>
-      <c r="E16" s="26" t="s">
+      <c r="D18" s="65"/>
+      <c r="E18" s="75" t="s">
         <v>99</v>
       </c>
-      <c r="F16" s="27"/>
-      <c r="G16" s="3" t="s">
+      <c r="F18" s="76"/>
+      <c r="G18" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="I16" s="46" t="s">
-        <v>78</v>
-      </c>
-      <c r="J16" s="46"/>
-      <c r="K16" s="46"/>
-      <c r="L16" s="46"/>
-      <c r="M16" s="46"/>
-      <c r="N16" s="46"/>
-    </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B17" s="2" t="s">
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B19" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C19" s="65" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="25"/>
-      <c r="E17" s="26" t="s">
+      <c r="D19" s="65"/>
+      <c r="E19" s="75" t="s">
         <v>100</v>
       </c>
-      <c r="F17" s="27"/>
-      <c r="G17" s="3" t="s">
+      <c r="F19" s="76"/>
+      <c r="G19" s="3" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B18" s="8" t="s">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B20" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="C20" s="65" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="25"/>
-      <c r="E18" s="26" t="s">
+      <c r="D20" s="65"/>
+      <c r="E20" s="75" t="s">
         <v>101</v>
       </c>
-      <c r="F18" s="27"/>
-      <c r="G18" s="3" t="s">
+      <c r="F20" s="76"/>
+      <c r="G20" s="3" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B19" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C19" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="D19" s="25"/>
-      <c r="E19" s="26" t="s">
-        <v>102</v>
-      </c>
-      <c r="F19" s="27"/>
-      <c r="G19" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B20" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C20" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="D20" s="25"/>
-      <c r="E20" s="26" t="s">
-        <v>103</v>
-      </c>
-      <c r="F20" s="27"/>
-      <c r="G20" s="3" t="s">
+      <c r="I20" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
+      <c r="M20" s="30"/>
+      <c r="N20" s="30"/>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B22" s="80" t="s">
         <v>111</v>
       </c>
-      <c r="I20" s="40" t="s">
-        <v>114</v>
-      </c>
-      <c r="J20" s="40"/>
-      <c r="K20" s="40"/>
-      <c r="L20" s="40"/>
-      <c r="M20" s="40"/>
-      <c r="N20" s="40"/>
-    </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B22" s="78" t="s">
-        <v>113</v>
-      </c>
-      <c r="C22" s="78"/>
-      <c r="D22" s="78"/>
-      <c r="E22" s="78"/>
-      <c r="F22" s="78"/>
-      <c r="G22" s="78"/>
-    </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="C22" s="80"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="80"/>
+      <c r="F22" s="80"/>
+      <c r="G22" s="80"/>
+      <c r="I22" s="102" t="s">
+        <v>153</v>
+      </c>
+      <c r="J22" s="102"/>
+      <c r="K22" s="102" t="s">
+        <v>154</v>
+      </c>
+      <c r="L22" s="102"/>
+      <c r="M22" s="102" t="s">
+        <v>155</v>
+      </c>
+      <c r="N22" s="102"/>
+      <c r="O22" s="102" t="s">
+        <v>156</v>
+      </c>
+      <c r="P22" s="102"/>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
-    </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="I23" s="71" t="s">
+        <v>157</v>
+      </c>
+      <c r="J23" s="71"/>
+      <c r="K23" s="70">
+        <v>22</v>
+      </c>
+      <c r="L23" s="70"/>
+      <c r="M23" s="58"/>
+      <c r="N23" s="59"/>
+      <c r="O23" s="58"/>
+      <c r="P23" s="59"/>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B24" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="C24" s="77"/>
-      <c r="D24" s="77"/>
-      <c r="E24" s="77"/>
-      <c r="F24" s="77"/>
-      <c r="G24" s="77"/>
-    </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+      <c r="C24" s="79"/>
+      <c r="D24" s="79"/>
+      <c r="E24" s="79"/>
+      <c r="F24" s="79"/>
+      <c r="G24" s="79"/>
+      <c r="I24" s="71" t="s">
+        <v>158</v>
+      </c>
+      <c r="J24" s="71"/>
+      <c r="K24" s="105">
+        <v>72</v>
+      </c>
+      <c r="L24" s="106"/>
+      <c r="M24" s="58"/>
+      <c r="N24" s="59"/>
+      <c r="O24" s="58"/>
+      <c r="P24" s="59"/>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="I25" s="71" t="s">
+        <v>159</v>
+      </c>
+      <c r="J25" s="71"/>
+      <c r="K25" s="105">
+        <v>150</v>
+      </c>
+      <c r="L25" s="106"/>
+      <c r="M25" s="58"/>
+      <c r="N25" s="59"/>
+      <c r="O25" s="58"/>
+      <c r="P25" s="59"/>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
@@ -3043,19 +3440,168 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
     </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="I27" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="J27" s="30"/>
+      <c r="K27" s="30"/>
+      <c r="L27" s="30"/>
+      <c r="M27" s="30"/>
+      <c r="N27" s="30"/>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="I29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="M29" s="107" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="I30" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K30" s="6">
+        <v>0</v>
+      </c>
+      <c r="L30" s="108">
+        <v>0.7</v>
+      </c>
+      <c r="M30" s="109">
+        <f>K30*L30</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="I31" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="K31" s="6">
+        <v>3.99</v>
+      </c>
+      <c r="L31" s="108">
+        <v>0.2</v>
+      </c>
+      <c r="M31" s="109">
+        <f t="shared" ref="M31:M34" si="0">K31*L31</f>
+        <v>0.79800000000000004</v>
+      </c>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="I32" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="K32" s="6">
+        <v>8.99</v>
+      </c>
+      <c r="L32" s="108">
+        <v>0.05</v>
+      </c>
+      <c r="M32" s="109">
+        <f t="shared" si="0"/>
+        <v>0.44950000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="9:13" x14ac:dyDescent="0.3">
+      <c r="I33" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K33" s="6">
+        <v>24.99</v>
+      </c>
+      <c r="L33" s="108">
+        <v>0.01</v>
+      </c>
+      <c r="M33" s="109">
+        <f t="shared" si="0"/>
+        <v>0.24989999999999998</v>
+      </c>
+    </row>
+    <row r="34" spans="9:13" x14ac:dyDescent="0.3">
+      <c r="I34" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K34" s="6">
+        <v>4</v>
+      </c>
+      <c r="L34" s="108">
+        <v>0.04</v>
+      </c>
+      <c r="M34" s="109">
+        <f t="shared" si="0"/>
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="35" spans="9:13" x14ac:dyDescent="0.3">
+      <c r="I35" s="90" t="s">
+        <v>163</v>
+      </c>
+      <c r="J35" s="90"/>
+      <c r="K35" s="112">
+        <f>SUM(K30:K34)</f>
+        <v>41.97</v>
+      </c>
+      <c r="L35" s="110">
+        <f>SUM(L30:L34)</f>
+        <v>1</v>
+      </c>
+      <c r="M35" s="111">
+        <f>SUM(M30:M34)</f>
+        <v>1.6574</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="I13:N13"/>
-    <mergeCell ref="I14:N14"/>
-    <mergeCell ref="I15:N15"/>
-    <mergeCell ref="I16:N16"/>
-    <mergeCell ref="B2:G5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B10:G10"/>
-    <mergeCell ref="I12:N12"/>
-    <mergeCell ref="B12:G12"/>
+  <mergeCells count="48">
+    <mergeCell ref="I27:N27"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="O23:P23"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="I20:N20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="M22:N22"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="E16:F16"/>
@@ -3068,13 +3614,17 @@
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="I20:N20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="I13:N13"/>
+    <mergeCell ref="I14:N14"/>
+    <mergeCell ref="I15:N15"/>
+    <mergeCell ref="I16:N16"/>
+    <mergeCell ref="B2:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="I12:N12"/>
+    <mergeCell ref="B12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -3090,190 +3640,180 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.21875" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" customWidth="1"/>
     <col min="8" max="8" width="2.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="32"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="36"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B3" s="33"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="35"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="39"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B4" s="33"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="35"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="39"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B5" s="33"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="35"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="39"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="38"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="42"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="41"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="44"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="44"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="47"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B12" s="74" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
+      <c r="F12" s="74"/>
+      <c r="G12" s="74"/>
+      <c r="I12" s="74" t="s">
         <v>115</v>
       </c>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="28" t="s">
+      <c r="J12" s="74"/>
+      <c r="K12" s="74"/>
+      <c r="L12" s="74"/>
+      <c r="M12" s="74"/>
+      <c r="N12" s="74"/>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B13" s="69" t="s">
         <v>116</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="I12" s="28" t="s">
+      <c r="C13" s="69"/>
+      <c r="D13" s="69" t="s">
         <v>117</v>
       </c>
-      <c r="J12" s="28"/>
-      <c r="K12" s="28"/>
-      <c r="L12" s="28"/>
-      <c r="M12" s="28"/>
-      <c r="N12" s="28"/>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="29" t="s">
+      <c r="E13" s="69"/>
+      <c r="F13" s="69" t="s">
         <v>118</v>
       </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29" t="s">
+      <c r="G13" s="69"/>
+      <c r="I13" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B14" s="65" t="s">
         <v>119</v>
       </c>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29" t="s">
+      <c r="C14" s="65"/>
+      <c r="D14" s="75"/>
+      <c r="E14" s="76"/>
+      <c r="F14" s="75"/>
+      <c r="G14" s="76"/>
+      <c r="I14" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B15" s="65" t="s">
         <v>120</v>
       </c>
-      <c r="G13" s="29"/>
-      <c r="I13" t="s">
+      <c r="C15" s="65"/>
+      <c r="D15" s="75"/>
+      <c r="E15" s="76"/>
+      <c r="F15" s="75"/>
+      <c r="G15" s="76"/>
+      <c r="I15" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B16" s="65" t="s">
+        <v>121</v>
+      </c>
+      <c r="C16" s="65"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="76"/>
+      <c r="F16" s="75"/>
+      <c r="G16" s="76"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17" s="65" t="s">
+        <v>122</v>
+      </c>
+      <c r="C17" s="65"/>
+      <c r="D17" s="75"/>
+      <c r="E17" s="76"/>
+      <c r="F17" s="75"/>
+      <c r="G17" s="76"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B18" s="65" t="s">
+        <v>123</v>
+      </c>
+      <c r="C18" s="65"/>
+      <c r="D18" s="75"/>
+      <c r="E18" s="76"/>
+      <c r="F18" s="75"/>
+      <c r="G18" s="76"/>
+      <c r="I18" t="s">
         <v>126</v>
-      </c>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="25" t="s">
-        <v>121</v>
-      </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="27"/>
-      <c r="I14" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="C15" s="25"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="27"/>
-      <c r="I15" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B16" s="25" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="25"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="27"/>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B17" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="C17" s="25"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="27"/>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B18" s="25" t="s">
-        <v>125</v>
-      </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="27"/>
-      <c r="I18" t="s">
-        <v>128</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B2:G5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B10:G10"/>
-    <mergeCell ref="I12:N12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B12:G12"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="F14:G14"/>
@@ -3288,6 +3828,17 @@
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
+    <mergeCell ref="I12:N12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B2:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B10:G10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3304,178 +3855,178 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="32"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="36"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B3" s="33"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="35"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="39"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B4" s="33"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="35"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="39"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B5" s="33"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="35"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="39"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="38"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="42"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="41"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="44"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="44"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="47"/>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="40" t="s">
-        <v>130</v>
-      </c>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
+      <c r="B11" s="30" t="s">
+        <v>128</v>
+      </c>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B12" s="95" t="s">
-        <v>131</v>
-      </c>
-      <c r="C12" s="96"/>
+      <c r="B12" s="86" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12" s="87"/>
       <c r="D12" s="14"/>
       <c r="E12" s="10"/>
-      <c r="F12" s="97">
+      <c r="F12" s="88">
         <f>Costs!F19</f>
         <v>75</v>
       </c>
-      <c r="G12" s="98"/>
+      <c r="G12" s="89"/>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B13" s="90" t="s">
-        <v>132</v>
-      </c>
-      <c r="C13" s="75"/>
-      <c r="F13" s="91">
+      <c r="B13" s="81" t="s">
+        <v>130</v>
+      </c>
+      <c r="C13" s="61"/>
+      <c r="F13" s="82">
         <f>Costs!F32</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="92"/>
+        <v>43.8</v>
+      </c>
+      <c r="G13" s="83"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B14" s="90" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14" s="75"/>
+      <c r="B14" s="81" t="s">
+        <v>131</v>
+      </c>
+      <c r="C14" s="61"/>
       <c r="F14" s="16"/>
       <c r="G14" s="17"/>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B15" s="15" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C15" s="7"/>
       <c r="F15" s="16"/>
       <c r="G15" s="17"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B16" s="93" t="s">
-        <v>134</v>
-      </c>
-      <c r="C16" s="94"/>
-      <c r="D16" s="94"/>
+      <c r="B16" s="84" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" s="85"/>
+      <c r="D16" s="85"/>
       <c r="E16" s="12"/>
       <c r="F16" s="18"/>
       <c r="G16" s="19"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B17" s="84"/>
-      <c r="C17" s="84"/>
-      <c r="D17" s="84"/>
+      <c r="B17" s="93"/>
+      <c r="C17" s="93"/>
+      <c r="D17" s="93"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B18" s="73" t="s">
+      <c r="B18" s="63" t="s">
+        <v>133</v>
+      </c>
+      <c r="C18" s="63"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B19" s="94" t="s">
+        <v>134</v>
+      </c>
+      <c r="C19" s="95"/>
+      <c r="D19" s="90" t="s">
+        <v>138</v>
+      </c>
+      <c r="E19" s="90"/>
+      <c r="F19" s="90"/>
+      <c r="G19" s="91"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B20" s="96" t="s">
         <v>135</v>
       </c>
-      <c r="C18" s="73"/>
-      <c r="D18" s="73"/>
-      <c r="E18" s="73"/>
-      <c r="F18" s="73"/>
-      <c r="G18" s="73"/>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B19" s="85" t="s">
-        <v>136</v>
-      </c>
-      <c r="C19" s="86"/>
-      <c r="D19" s="81" t="s">
-        <v>140</v>
-      </c>
-      <c r="E19" s="81"/>
-      <c r="F19" s="81"/>
-      <c r="G19" s="82"/>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B20" s="87" t="s">
-        <v>137</v>
-      </c>
-      <c r="C20" s="46"/>
+      <c r="C20" s="32"/>
       <c r="D20" s="48"/>
       <c r="E20" s="48"/>
       <c r="F20" s="48"/>
-      <c r="G20" s="83"/>
+      <c r="G20" s="92"/>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B21" s="87" t="s">
-        <v>138</v>
-      </c>
-      <c r="C21" s="46"/>
+      <c r="B21" s="96" t="s">
+        <v>136</v>
+      </c>
+      <c r="C21" s="32"/>
       <c r="G21" s="11"/>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B22" s="88" t="s">
-        <v>139</v>
-      </c>
-      <c r="C22" s="89"/>
+      <c r="B22" s="97" t="s">
+        <v>137</v>
+      </c>
+      <c r="C22" s="98"/>
       <c r="D22" s="12"/>
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
@@ -3487,6 +4038,15 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="F13:G13"/>
@@ -3498,15 +4058,6 @@
     <mergeCell ref="B11:G11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="F12:G12"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>